<commit_message>
Supply cost fixes to align with PIER2.0+Rumi
</commit_message>
<xml_diff>
--- a/electricity_fiveZ_8736_2p_nziShadow_dev/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
+++ b/electricity_fiveZ_8736_2p_nziShadow_dev/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apascale\OneDrive - Princeton University\Documents\GitHub\NZx_caseDev_MacroEP\electricity_fiveZ_8736_2p_nziShadow_dev\viz_compare_info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEAB39F1-1C62-4FA0-85FB-0EFBBBB41746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99907D40-1908-4110-AB42-85CE9DBCB50D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0C04E4D0-5751-44E6-BC3B-AD203EDB8BF9}"/>
   </bookViews>
@@ -1028,7 +1028,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -1039,6 +1039,7 @@
     <numFmt numFmtId="170" formatCode="0.000000"/>
     <numFmt numFmtId="171" formatCode="0.0000000"/>
     <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="173" formatCode="0.0000"/>
   </numFmts>
   <fonts count="28" x14ac:knownFonts="1">
     <font>
@@ -1836,7 +1837,7 @@
     <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
@@ -2100,6 +2101,7 @@
     <xf numFmtId="2" fontId="0" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="43" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3086,6 +3088,8 @@
     <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="12" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -3393,8 +3397,8 @@
         <v>2.8103758044980376</v>
       </c>
       <c r="Z6" s="2">
-        <f>Carriers!H$28*1000</f>
-        <v>1942097.6230000001</v>
+        <f>Carriers!H$3*1000</f>
+        <v>1871873.679</v>
       </c>
       <c r="AA6" s="2">
         <f>Carriers!G$3*277800</f>
@@ -3402,11 +3406,11 @@
       </c>
       <c r="AB6">
         <f>Z6/AA6</f>
-        <v>0.40628325241905094</v>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AC6">
         <f>AB6*Y6</f>
-        <v>1.1418086223712696</v>
+        <v>1.1005221783704484</v>
       </c>
       <c r="AD6" t="s">
         <v>319</v>
@@ -3415,19 +3419,19 @@
         <v>13</v>
       </c>
       <c r="AF6" s="4">
-        <f>11751.5992748699</f>
-        <v>11751.599274869899</v>
+        <f>P6/1000</f>
+        <v>11.7515992748699</v>
       </c>
       <c r="AG6">
         <v>3</v>
       </c>
       <c r="AH6">
-        <f>AG6*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG6*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI6" s="4">
-        <f t="shared" ref="AI6:AI22" si="0">AF6-AH6</f>
-        <v>8034.846530456527</v>
+        <f>AF6-AH6</f>
+        <v>8.0348465304565266</v>
       </c>
       <c r="AJ6">
         <v>10</v>
@@ -3436,12 +3440,12 @@
         <v>0.105</v>
       </c>
       <c r="AL6">
-        <f t="shared" ref="AL6:AL22" si="1">AK6/(1-(1+AK6)^-AJ6)</f>
+        <f>AK6/(1-(1+AK6)^-AJ6)</f>
         <v>0.16625732062625342</v>
       </c>
-      <c r="AM6" s="4">
-        <f t="shared" ref="AM6:AM22" si="2">AI6/AL6</f>
-        <v>48327.775884942042</v>
+      <c r="AM6" s="125">
+        <f>AI6/AL6</f>
+        <v>48.327775884942035</v>
       </c>
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.25">
@@ -3500,7 +3504,7 @@
         <v>7.8507860294473842E-5</v>
       </c>
       <c r="T7" s="1">
-        <f t="shared" ref="T7:T22" si="3">J7/Y7</f>
+        <f t="shared" ref="T7:T22" si="0">J7/Y7</f>
         <v>2.3484403720799997E-2</v>
       </c>
       <c r="U7" t="s">
@@ -3516,12 +3520,12 @@
         <v>1871.873679</v>
       </c>
       <c r="Y7" s="1">
-        <f t="shared" ref="Y7:Y18" si="4">1/H7/(1-J7)</f>
+        <f t="shared" ref="Y7:Y18" si="1">1/H7/(1-J7)</f>
         <v>2.8103758044980376</v>
       </c>
       <c r="Z7" s="2">
-        <f>Carriers!H$28*1000</f>
-        <v>1942097.6230000001</v>
+        <f>Carriers!H$3*1000</f>
+        <v>1871873.679</v>
       </c>
       <c r="AA7" s="2">
         <f>Carriers!G$3*277800</f>
@@ -3529,11 +3533,11 @@
       </c>
       <c r="AB7">
         <f>Z7/AA7</f>
-        <v>0.40628325241905094</v>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AC7">
-        <f t="shared" ref="AC7:AC13" si="5">AB7</f>
-        <v>0.40628325241905094</v>
+        <f t="shared" ref="AC7:AC13" si="2">AB7</f>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AD7" t="s">
         <v>319</v>
@@ -3542,19 +3546,19 @@
         <v>10</v>
       </c>
       <c r="AF7" s="4">
-        <f>26148.8463751508</f>
-        <v>26148.846375150799</v>
+        <f t="shared" ref="AF7:AF18" si="3">P7/1000</f>
+        <v>26.1488463751508</v>
       </c>
       <c r="AG7">
         <v>3</v>
       </c>
       <c r="AH7">
-        <f>AG7*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG7*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI7" s="4">
-        <f t="shared" si="0"/>
-        <v>22432.093630737425</v>
+        <f t="shared" ref="AI7:AI22" si="4">AF7-AH7</f>
+        <v>22.432093630737427</v>
       </c>
       <c r="AJ7">
         <v>10</v>
@@ -3563,12 +3567,12 @@
         <v>0.105</v>
       </c>
       <c r="AL7">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="AL7:AL22" si="5">AK7/(1-(1+AK7)^-AJ7)</f>
         <v>0.16625732062625342</v>
       </c>
-      <c r="AM7" s="4">
-        <f t="shared" si="2"/>
-        <v>134923.94528097074</v>
+      <c r="AM7" s="125">
+        <f t="shared" ref="AM7:AM22" si="6">AI7/AL7</f>
+        <v>134.92394528097074</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.25">
@@ -3627,7 +3631,7 @@
         <v>7.8507860294473842E-5</v>
       </c>
       <c r="T8" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>2.3484403720799997E-2</v>
       </c>
       <c r="W8">
@@ -3637,24 +3641,24 @@
         <v>1871.873679</v>
       </c>
       <c r="Y8" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>2.8103758044980376</v>
       </c>
       <c r="Z8" s="2">
-        <f>Carriers!H$28*1000</f>
-        <v>1942097.6230000001</v>
+        <f>Carriers!H$3*1000</f>
+        <v>1871873.679</v>
       </c>
       <c r="AA8" s="2">
         <f>Carriers!G$3*277800</f>
         <v>4780156.7291700002</v>
       </c>
       <c r="AB8">
-        <f t="shared" ref="AB8:AB12" si="6">Z8/AA8</f>
-        <v>0.40628325241905094</v>
+        <f t="shared" ref="AB8:AB12" si="7">Z8/AA8</f>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AC8">
-        <f t="shared" si="5"/>
-        <v>0.40628325241905094</v>
+        <f t="shared" si="2"/>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AD8" t="s">
         <v>319</v>
@@ -3663,19 +3667,19 @@
         <v>11</v>
       </c>
       <c r="AF8" s="4">
-        <f>6514.90571684157</f>
-        <v>6514.9057168415702</v>
+        <f t="shared" si="3"/>
+        <v>6.5149057168415698</v>
       </c>
       <c r="AG8">
         <v>3</v>
       </c>
       <c r="AH8">
-        <f>AG8*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG8*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI8" s="4">
-        <f t="shared" si="0"/>
-        <v>2798.1529724281977</v>
+        <f t="shared" si="4"/>
+        <v>2.7981529724281975</v>
       </c>
       <c r="AJ8">
         <v>10</v>
@@ -3684,12 +3688,12 @@
         <v>0.105</v>
       </c>
       <c r="AL8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.16625732062625342</v>
       </c>
-      <c r="AM8" s="4">
-        <f t="shared" si="2"/>
-        <v>16830.254222119023</v>
+      <c r="AM8" s="125">
+        <f t="shared" si="6"/>
+        <v>16.83025422211902</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.25">
@@ -3748,7 +3752,7 @@
         <v>7.8507860294473842E-5</v>
       </c>
       <c r="T9" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>2.3484403720799997E-2</v>
       </c>
       <c r="W9">
@@ -3758,24 +3762,24 @@
         <v>1871.873679</v>
       </c>
       <c r="Y9" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>2.8103758044980376</v>
       </c>
       <c r="Z9" s="2">
-        <f>Carriers!H$28*1000</f>
-        <v>1942097.6230000001</v>
+        <f>Carriers!H$3*1000</f>
+        <v>1871873.679</v>
       </c>
       <c r="AA9" s="2">
         <f>Carriers!G$3*277800</f>
         <v>4780156.7291700002</v>
       </c>
       <c r="AB9">
-        <f t="shared" si="6"/>
-        <v>0.40628325241905094</v>
+        <f t="shared" si="7"/>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AC9">
-        <f t="shared" si="5"/>
-        <v>0.40628325241905094</v>
+        <f t="shared" si="2"/>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AD9" t="s">
         <v>319</v>
@@ -3784,19 +3788,19 @@
         <v>12</v>
       </c>
       <c r="AF9" s="4">
-        <f>5794.65159561365</f>
-        <v>5794.65159561365</v>
+        <f t="shared" si="3"/>
+        <v>5.79465159561365</v>
       </c>
       <c r="AG9">
         <v>3</v>
       </c>
       <c r="AH9">
-        <f>AG9*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG9*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI9" s="4">
-        <f t="shared" si="0"/>
-        <v>2077.8988512002775</v>
+        <f t="shared" si="4"/>
+        <v>2.0778988512002776</v>
       </c>
       <c r="AJ9">
         <v>10</v>
@@ -3805,12 +3809,12 @@
         <v>0.105</v>
       </c>
       <c r="AL9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.16625732062625342</v>
       </c>
-      <c r="AM9" s="4">
-        <f t="shared" si="2"/>
-        <v>12498.089367573748</v>
+      <c r="AM9" s="125">
+        <f t="shared" si="6"/>
+        <v>12.498089367573749</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.25">
@@ -3869,7 +3873,7 @@
         <v>7.8507860294473842E-5</v>
       </c>
       <c r="T10" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>2.3484403720799997E-2</v>
       </c>
       <c r="W10">
@@ -3879,24 +3883,24 @@
         <v>1871.873679</v>
       </c>
       <c r="Y10" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>2.8103758044980376</v>
       </c>
       <c r="Z10" s="2">
-        <f>Carriers!H$28*1000</f>
-        <v>1942097.6230000001</v>
+        <f>Carriers!H$3*1000</f>
+        <v>1871873.679</v>
       </c>
       <c r="AA10" s="2">
         <f>Carriers!G$3*277800</f>
         <v>4780156.7291700002</v>
       </c>
       <c r="AB10">
-        <f t="shared" si="6"/>
-        <v>0.40628325241905094</v>
+        <f t="shared" si="7"/>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AC10">
-        <f t="shared" si="5"/>
-        <v>0.40628325241905094</v>
+        <f t="shared" si="2"/>
+        <v>0.3915925324325133</v>
       </c>
       <c r="AD10" t="s">
         <v>319</v>
@@ -3905,19 +3909,19 @@
         <v>9</v>
       </c>
       <c r="AF10" s="4">
-        <f>5822.44460147077</f>
-        <v>5822.4446014707701</v>
+        <f t="shared" si="3"/>
+        <v>5.82244460147077</v>
       </c>
       <c r="AG10">
         <v>3</v>
       </c>
       <c r="AH10">
-        <f>AG10*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG10*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI10" s="4">
-        <f t="shared" si="0"/>
-        <v>2105.6918570573976</v>
+        <f t="shared" si="4"/>
+        <v>2.1056918570573977</v>
       </c>
       <c r="AJ10">
         <v>10</v>
@@ -3926,12 +3930,12 @@
         <v>0.105</v>
       </c>
       <c r="AL10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.16625732062625342</v>
       </c>
-      <c r="AM10" s="4">
-        <f t="shared" si="2"/>
-        <v>12665.257981577812</v>
+      <c r="AM10" s="125">
+        <f t="shared" si="6"/>
+        <v>12.665257981577813</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.25">
@@ -3948,19 +3952,19 @@
         <v>319</v>
       </c>
       <c r="AF11" s="4">
-        <f>13721031.29/1000</f>
-        <v>13721.031289999999</v>
+        <f>Q10/1000</f>
+        <v>13.721031289999999</v>
       </c>
       <c r="AG11" s="123">
         <v>3</v>
       </c>
       <c r="AH11">
-        <f>AG11*Conversions!$D$5*1000</f>
-        <v>3716.7527444133725</v>
+        <f>AG11*Conversions!$D$5</f>
+        <v>3.7167527444133723</v>
       </c>
       <c r="AI11" s="4">
-        <f t="shared" si="0"/>
-        <v>10004.278545586627</v>
+        <f t="shared" si="4"/>
+        <v>10.004278545586626</v>
       </c>
       <c r="AJ11">
         <v>40</v>
@@ -3969,12 +3973,12 @@
         <v>0.105</v>
       </c>
       <c r="AL11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.10697140835497033</v>
       </c>
-      <c r="AM11" s="4">
-        <f t="shared" si="2"/>
-        <v>93522.920745221607</v>
+      <c r="AM11" s="125">
+        <f t="shared" si="6"/>
+        <v>93.522920745221597</v>
       </c>
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.25">
@@ -4032,11 +4036,11 @@
         <v>0</v>
       </c>
       <c r="T12" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>7.9270773512000008E-3</v>
       </c>
       <c r="Y12" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>2.5229979617863072</v>
       </c>
       <c r="Z12" s="2">
@@ -4048,11 +4052,11 @@
         <v>12627065.572979493</v>
       </c>
       <c r="AB12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.23956670942401803</v>
       </c>
       <c r="AC12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v>0.23956670942401803</v>
       </c>
       <c r="AD12" t="str">
@@ -4060,19 +4064,19 @@
         <v>EG_CCGT</v>
       </c>
       <c r="AF12" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q12</f>
-        <v>8512.2278029999998</v>
+        <f t="shared" si="3"/>
+        <v>8.5122278027488392</v>
       </c>
       <c r="AG12">
         <v>2.9</v>
       </c>
       <c r="AH12">
-        <f>AG12*Conversions!$D$5*1000</f>
-        <v>3592.8609862662602</v>
+        <f>AG12*Conversions!$D$5</f>
+        <v>3.5928609862662602</v>
       </c>
       <c r="AI12" s="4">
-        <f t="shared" si="0"/>
-        <v>4919.3668167337401</v>
+        <f t="shared" si="4"/>
+        <v>4.9193668164825795</v>
       </c>
       <c r="AJ12">
         <v>25</v>
@@ -4081,12 +4085,12 @@
         <v>0.105</v>
       </c>
       <c r="AL12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11442931981310331</v>
       </c>
-      <c r="AM12" s="4">
-        <f t="shared" si="2"/>
-        <v>42990.440079242901</v>
+      <c r="AM12" s="125">
+        <f t="shared" si="6"/>
+        <v>42.990440077048</v>
       </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.25">
@@ -4144,11 +4148,11 @@
         <v>0</v>
       </c>
       <c r="T13" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>2.7789461171999997E-3</v>
       </c>
       <c r="Y13" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>3.5984864687033813</v>
       </c>
       <c r="Z13" s="2">
@@ -4160,11 +4164,11 @@
         <v>12627065.572979493</v>
       </c>
       <c r="AB13">
-        <f t="shared" ref="AB13" si="7">Z13/AA13</f>
+        <f t="shared" ref="AB13" si="8">Z13/AA13</f>
         <v>0.23956670942401803</v>
       </c>
       <c r="AC13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v>0.23956670942401803</v>
       </c>
       <c r="AD13" t="str">
@@ -4172,19 +4176,19 @@
         <v>EG_OCGT</v>
       </c>
       <c r="AF13" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q13</f>
-        <v>6679.7506490000005</v>
+        <f t="shared" si="3"/>
+        <v>6.6797506492714502</v>
       </c>
       <c r="AG13">
         <v>0.7</v>
       </c>
       <c r="AH13">
-        <f>AG13*Conversions!$D$5*1000</f>
-        <v>867.24230702978684</v>
+        <f>AG13*Conversions!$D$5</f>
+        <v>0.86724230702978689</v>
       </c>
       <c r="AI13" s="4">
-        <f t="shared" si="0"/>
-        <v>5812.5083419702132</v>
+        <f t="shared" si="4"/>
+        <v>5.8125083422416637</v>
       </c>
       <c r="AJ13">
         <v>25</v>
@@ -4193,12 +4197,12 @@
         <v>0.105</v>
       </c>
       <c r="AL13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11442931981310331</v>
       </c>
-      <c r="AM13" s="4">
-        <f t="shared" si="2"/>
-        <v>50795.620837943869</v>
+      <c r="AM13" s="125">
+        <f t="shared" si="6"/>
+        <v>50.795620840316076</v>
       </c>
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.25">
@@ -4256,11 +4260,11 @@
         <v>0</v>
       </c>
       <c r="T14" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>9.6179160000000014E-2</v>
       </c>
       <c r="Y14" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>1.1208249271463797</v>
       </c>
       <c r="AD14" t="str">
@@ -4268,19 +4272,19 @@
         <v>EG_PHWR</v>
       </c>
       <c r="AF14" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q14</f>
-        <v>20833.210350000001</v>
+        <f t="shared" si="3"/>
+        <v>20.833210347832701</v>
       </c>
       <c r="AG14">
         <v>4.3</v>
       </c>
       <c r="AH14">
-        <f>AG14*Conversions!$D$5*1000</f>
-        <v>5327.3456003258334</v>
+        <f>AG14*Conversions!$D$5</f>
+        <v>5.3273456003258337</v>
       </c>
       <c r="AI14" s="4">
-        <f t="shared" si="0"/>
-        <v>15505.864749674169</v>
+        <f t="shared" si="4"/>
+        <v>15.505864747506866</v>
       </c>
       <c r="AJ14">
         <v>40</v>
@@ -4289,12 +4293,12 @@
         <v>0.105</v>
       </c>
       <c r="AL14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.10697140835497033</v>
       </c>
-      <c r="AM14" s="4">
-        <f t="shared" si="2"/>
-        <v>144953.35705238194</v>
+      <c r="AM14" s="125">
+        <f t="shared" si="6"/>
+        <v>144.95335703212137</v>
       </c>
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.25">
@@ -4349,11 +4353,11 @@
         <v>0</v>
       </c>
       <c r="T15" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>4.7500000000000007E-2</v>
       </c>
       <c r="Y15" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>1.0526315789473684</v>
       </c>
       <c r="AD15" t="str">
@@ -4361,19 +4365,19 @@
         <v>EG_SMR</v>
       </c>
       <c r="AF15" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q15</f>
-        <v>35289.429389999998</v>
+        <f>Q15/1000</f>
+        <v>35.289429389999995</v>
       </c>
       <c r="AG15">
         <v>5</v>
       </c>
       <c r="AH15">
-        <f>AG15*Conversions!$D$5*1000</f>
-        <v>6194.5879073556207</v>
+        <f>AG15*Conversions!$D$5</f>
+        <v>6.1945879073556211</v>
       </c>
       <c r="AI15" s="4">
-        <f t="shared" si="0"/>
-        <v>29094.841482644377</v>
+        <f t="shared" si="4"/>
+        <v>29.094841482644373</v>
       </c>
       <c r="AJ15">
         <v>30</v>
@@ -4382,12 +4386,12 @@
         <v>0.105</v>
       </c>
       <c r="AL15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11052848152960514</v>
       </c>
-      <c r="AM15" s="4">
-        <f t="shared" si="2"/>
-        <v>263233.88397271431</v>
+      <c r="AM15" s="125">
+        <f t="shared" si="6"/>
+        <v>263.2338839727143</v>
       </c>
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.25">
@@ -4445,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="T16" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>6.0362173038229381E-3</v>
       </c>
       <c r="Y16" s="121">
@@ -4457,19 +4461,19 @@
         <v>EG_LH</v>
       </c>
       <c r="AF16" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q16</f>
-        <v>19631.81452</v>
+        <f t="shared" si="3"/>
+        <v>19.631814520722802</v>
       </c>
       <c r="AG16">
         <v>4.4000000000000004</v>
       </c>
       <c r="AH16">
-        <f>AG16*Conversions!$D$5*1000</f>
-        <v>5451.2373584729476</v>
+        <f>AG16*Conversions!$D$5</f>
+        <v>5.4512373584729472</v>
       </c>
       <c r="AI16" s="4">
-        <f t="shared" si="0"/>
-        <v>14180.577161527053</v>
+        <f t="shared" si="4"/>
+        <v>14.180577162249854</v>
       </c>
       <c r="AJ16">
         <v>40</v>
@@ -4478,12 +4482,12 @@
         <v>0.105</v>
       </c>
       <c r="AL16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.10697140835497033</v>
       </c>
-      <c r="AM16" s="4">
-        <f t="shared" si="2"/>
-        <v>132564.18121065304</v>
+      <c r="AM16" s="125">
+        <f t="shared" si="6"/>
+        <v>132.56418121741001</v>
       </c>
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.25">
@@ -4541,7 +4545,7 @@
         <v>0</v>
       </c>
       <c r="T17" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>1.0101010101010102E-2</v>
       </c>
       <c r="Y17" s="121">
@@ -4553,20 +4557,20 @@
         <v>EG_SH</v>
       </c>
       <c r="AF17" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q17</f>
-        <v>11825.348759999999</v>
+        <f t="shared" si="3"/>
+        <v>11.825348755495598</v>
       </c>
       <c r="AG17">
         <f>2.4</f>
         <v>2.4</v>
       </c>
       <c r="AH17">
-        <f>AG17*Conversions!$D$5*1000</f>
-        <v>2973.402195530698</v>
+        <f>AG17*Conversions!$D$5</f>
+        <v>2.973402195530698</v>
       </c>
       <c r="AI17" s="4">
-        <f t="shared" si="0"/>
-        <v>8851.9465644693009</v>
+        <f t="shared" si="4"/>
+        <v>8.851946559964901</v>
       </c>
       <c r="AJ17">
         <v>35</v>
@@ -4575,12 +4579,12 @@
         <v>8.3500000000000005E-2</v>
       </c>
       <c r="AL17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>8.8866958914066166E-2</v>
       </c>
-      <c r="AM17" s="4">
-        <f t="shared" si="2"/>
-        <v>99608.973600965488</v>
+      <c r="AM17" s="125">
+        <f t="shared" si="6"/>
+        <v>99.608973550278478</v>
       </c>
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.25">
@@ -4638,11 +4642,11 @@
         <v>0</v>
       </c>
       <c r="T18" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>2.1496130730000004E-2</v>
       </c>
       <c r="Y18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>4.6519999927447406</v>
       </c>
       <c r="Z18" s="2">
@@ -4654,7 +4658,7 @@
         <v>3791683.3103999998</v>
       </c>
       <c r="AB18">
-        <f t="shared" ref="AB18" si="8">Z18/AA18</f>
+        <f t="shared" ref="AB18" si="9">Z18/AA18</f>
         <v>0.43686050558511857</v>
       </c>
       <c r="AC18">
@@ -4666,19 +4670,19 @@
         <v>EG_BIOMASS</v>
       </c>
       <c r="AF18" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q18</f>
-        <v>7713.4572400000006</v>
+        <f t="shared" si="3"/>
+        <v>7.7134572396533407</v>
       </c>
       <c r="AG18" s="118">
         <v>1</v>
       </c>
       <c r="AH18">
-        <f>AG18*Conversions!$D$5*1000</f>
-        <v>1238.9175814711241</v>
+        <f>AG18*Conversions!$D$5</f>
+        <v>1.2389175814711242</v>
       </c>
       <c r="AI18" s="4">
-        <f t="shared" si="0"/>
-        <v>6474.5396585288763</v>
+        <f t="shared" si="4"/>
+        <v>6.4745396581822163</v>
       </c>
       <c r="AJ18">
         <v>20</v>
@@ -4687,12 +4691,12 @@
         <v>8.3500000000000005E-2</v>
       </c>
       <c r="AL18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.10451929579519206</v>
       </c>
-      <c r="AM18" s="4">
-        <f t="shared" si="2"/>
-        <v>61945.879076872887</v>
+      <c r="AM18" s="125">
+        <f t="shared" si="6"/>
+        <v>61.945879073556178</v>
       </c>
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.25">
@@ -4750,7 +4754,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>0.01</v>
       </c>
       <c r="Y19" s="119">
@@ -4761,19 +4765,19 @@
         <v>EG_SOLARGM</v>
       </c>
       <c r="AF19" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q19</f>
-        <v>5439.7058559999996</v>
+        <f>Q19/1000</f>
+        <v>5.4397058559999998</v>
       </c>
       <c r="AG19">
         <v>0.35</v>
       </c>
       <c r="AH19">
-        <f>AG19*Conversions!$D$5*1000</f>
-        <v>433.62115351489342</v>
+        <f>AG19*Conversions!$D$5</f>
+        <v>0.43362115351489344</v>
       </c>
       <c r="AI19" s="4">
-        <f t="shared" si="0"/>
-        <v>5006.0847024851064</v>
+        <f>AF19-AH19</f>
+        <v>5.0060847024851061</v>
       </c>
       <c r="AJ19">
         <v>25</v>
@@ -4782,12 +4786,12 @@
         <v>0.105</v>
       </c>
       <c r="AL19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11442931981310331</v>
       </c>
-      <c r="AM19" s="4">
-        <f t="shared" si="2"/>
-        <v>43748.269330461051</v>
+      <c r="AM19" s="125">
+        <f t="shared" si="6"/>
+        <v>43.748269330461049</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.25">
@@ -4845,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Y20" s="119">
@@ -4856,19 +4860,19 @@
         <v>EG_SOLARRF</v>
       </c>
       <c r="AF20" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q20</f>
-        <v>5362.1338370000003</v>
+        <f>Q20/1000</f>
+        <v>5.362133837</v>
       </c>
       <c r="AG20">
         <v>0.51</v>
       </c>
       <c r="AH20">
-        <f>AG20*Conversions!$D$5*1000</f>
-        <v>631.84796655027333</v>
+        <f>AG20*Conversions!$D$5</f>
+        <v>0.63184796655027331</v>
       </c>
       <c r="AI20" s="4">
-        <f t="shared" si="0"/>
-        <v>4730.2858704497266</v>
+        <f t="shared" si="4"/>
+        <v>4.7302858704497268</v>
       </c>
       <c r="AJ20">
         <v>25</v>
@@ -4877,12 +4881,12 @@
         <v>0.104</v>
       </c>
       <c r="AL20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11357300490974749</v>
       </c>
-      <c r="AM20" s="4">
-        <f t="shared" si="2"/>
-        <v>41649.737754220027</v>
+      <c r="AM20" s="125">
+        <f t="shared" si="6"/>
+        <v>41.649737754220027</v>
       </c>
     </row>
     <row r="21" spans="1:39" x14ac:dyDescent="0.25">
@@ -4940,7 +4944,7 @@
         <v>0</v>
       </c>
       <c r="T21" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="Y21" s="119">
@@ -4951,19 +4955,19 @@
         <v>EG_WINDON</v>
       </c>
       <c r="AF21" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q21</f>
-        <v>10586.964460000001</v>
+        <f>Q21/1000</f>
+        <v>10.586964460000001</v>
       </c>
       <c r="AG21">
         <v>0.68</v>
       </c>
       <c r="AH21">
-        <f>AG21*Conversions!$D$5*1000</f>
-        <v>842.46395540036451</v>
+        <f>AG21*Conversions!$D$5</f>
+        <v>0.84246395540036456</v>
       </c>
       <c r="AI21" s="4">
-        <f t="shared" si="0"/>
-        <v>9744.5005045996368</v>
+        <f t="shared" si="4"/>
+        <v>9.7445005045996353</v>
       </c>
       <c r="AJ21">
         <v>25</v>
@@ -4972,12 +4976,12 @@
         <v>0.105</v>
       </c>
       <c r="AL21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.11442931981310331</v>
       </c>
-      <c r="AM21" s="4">
-        <f t="shared" si="2"/>
-        <v>85157.375054883392</v>
+      <c r="AM21" s="125">
+        <f t="shared" si="6"/>
+        <v>85.157375054883374</v>
       </c>
     </row>
     <row r="22" spans="1:39" x14ac:dyDescent="0.25">
@@ -5032,7 +5036,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="Y22" s="119">
@@ -5043,19 +5047,19 @@
         <v>EG_WINDOFF</v>
       </c>
       <c r="AF22" s="4">
-        <f>ECT_EfficiencyCostMaxAnnualUF!Q22</f>
-        <v>34540.361669999998</v>
+        <f>Q22/1000</f>
+        <v>34.540361669999996</v>
       </c>
       <c r="AG22">
         <v>6.7</v>
       </c>
       <c r="AH22">
-        <f>AG22*Conversions!$D$5*1000</f>
-        <v>8300.7477958565323</v>
+        <f>AG22*Conversions!$D$5</f>
+        <v>8.3007477958565321</v>
       </c>
       <c r="AI22" s="4">
-        <f t="shared" si="0"/>
-        <v>26239.613874143466</v>
+        <f t="shared" si="4"/>
+        <v>26.239613874143465</v>
       </c>
       <c r="AJ22">
         <v>25</v>
@@ -5064,12 +5068,12 @@
         <v>0.112</v>
       </c>
       <c r="AL22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0.12047788778229078</v>
       </c>
-      <c r="AM22" s="4">
-        <f t="shared" si="2"/>
-        <v>217796.09816499843</v>
+      <c r="AM22" s="125">
+        <f t="shared" si="6"/>
+        <v>217.79609816499843</v>
       </c>
     </row>
     <row r="25" spans="1:39" x14ac:dyDescent="0.25">
@@ -5127,37 +5131,37 @@
     </row>
     <row r="33" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M33">
-        <f t="shared" ref="M33:M38" si="9">$M$26</f>
+        <f t="shared" ref="M33:M38" si="10">$M$26</f>
         <v>0.95</v>
       </c>
     </row>
     <row r="34" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M34">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.95</v>
       </c>
     </row>
     <row r="35" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M35">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.95</v>
       </c>
     </row>
     <row r="36" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M36">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.95</v>
       </c>
     </row>
     <row r="37" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M37">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.95</v>
       </c>
     </row>
     <row r="38" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M38">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.95</v>
       </c>
     </row>
@@ -9072,34 +9076,34 @@
         <v>157</v>
       </c>
       <c r="G7" s="16"/>
-      <c r="H7" s="125" t="s">
+      <c r="H7" s="126" t="s">
         <v>158</v>
       </c>
-      <c r="I7" s="125"/>
-      <c r="J7" s="125" t="s">
+      <c r="I7" s="126"/>
+      <c r="J7" s="126" t="s">
         <v>159</v>
       </c>
-      <c r="K7" s="125"/>
-      <c r="L7" s="125" t="s">
+      <c r="K7" s="126"/>
+      <c r="L7" s="126" t="s">
         <v>160</v>
       </c>
-      <c r="M7" s="125"/>
-      <c r="N7" s="125" t="s">
+      <c r="M7" s="126"/>
+      <c r="N7" s="126" t="s">
         <v>161</v>
       </c>
-      <c r="O7" s="125"/>
-      <c r="P7" s="125" t="s">
+      <c r="O7" s="126"/>
+      <c r="P7" s="126" t="s">
         <v>162</v>
       </c>
-      <c r="Q7" s="125"/>
-      <c r="R7" s="125" t="s">
+      <c r="Q7" s="126"/>
+      <c r="R7" s="126" t="s">
         <v>163</v>
       </c>
-      <c r="S7" s="125"/>
-      <c r="T7" s="125" t="s">
+      <c r="S7" s="126"/>
+      <c r="T7" s="126" t="s">
         <v>164</v>
       </c>
-      <c r="U7" s="125"/>
+      <c r="U7" s="126"/>
       <c r="V7" s="18"/>
       <c r="W7" s="18"/>
       <c r="X7" s="18"/>

</xml_diff>

<commit_message>
Fix y-axis label in readme image
</commit_message>
<xml_diff>
--- a/electricity_fiveZ_8736_2p_nziShadow_dev/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
+++ b/electricity_fiveZ_8736_2p_nziShadow_dev/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apascale\OneDrive - Princeton University\Documents\GitHub\NZx_caseDev_MacroEP\electricity_fiveZ_8736_2p_nziShadow_dev\viz_compare_info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99907D40-1908-4110-AB42-85CE9DBCB50D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACD7E97-B363-4552-9629-E999547D0EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0C04E4D0-5751-44E6-BC3B-AD203EDB8BF9}"/>
   </bookViews>
@@ -3397,8 +3397,8 @@
         <v>2.8103758044980376</v>
       </c>
       <c r="Z6" s="2">
-        <f>Carriers!H$3*1000</f>
-        <v>1871873.679</v>
+        <f>Carriers!H$28*1000</f>
+        <v>1942097.6230000001</v>
       </c>
       <c r="AA6" s="2">
         <f>Carriers!G$3*277800</f>
@@ -3406,11 +3406,11 @@
       </c>
       <c r="AB6">
         <f>Z6/AA6</f>
-        <v>0.3915925324325133</v>
+        <v>0.40628325241905094</v>
       </c>
       <c r="AC6">
         <f>AB6*Y6</f>
-        <v>1.1005221783704484</v>
+        <v>1.1418086223712696</v>
       </c>
       <c r="AD6" t="s">
         <v>319</v>

</xml_diff>